<commit_message>
Rework deck model docs: portrait SBS, measured anchors, customer slot names, side positions, pick-list sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X1RNxQHa1nUuDBKRsS4C3g
</commit_message>
<xml_diff>
--- a/docs/labot_zadani_parametry.xlsx
+++ b/docs/labot_zadani_parametry.xlsx
@@ -16,6 +16,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_Kvalita" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_Run" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8_Pipety" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_Konfigurace" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Pick_list" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -471,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -521,7 +523,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2_Deck       – sloty (3×2 SBS + 3 přední + 3 zadní úzké, předsazená řada), rozměry a omezení</t>
+          <t>2_Deck       – sloty A1–B3 (SBS na výšku), C1–C3 a 1–3 (úzké), L/R (boční), rozměry a omezení</t>
         </is>
       </c>
     </row>
@@ -568,23 +570,1029 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>9_Konfigurace – obsah slotů pro 12,5 µL a 300 µL pipetu (předvyplněno z vaší tabulky)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>10_Pick_list – cherry-picking / pooling / repliky jako seznam přenosů</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>Pojmy: správnost (trueness) = systematická odchylka od nominálního objemu v % nebo µL;</t>
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>přesnost (precision) = náhodná odchylka, CV v %. Vyplňte pro každou třídu kroku (list 6).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Slot</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Konfigurace s pipetou 12,5 µL (z tabulky zákazníka)</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Konfigurace s pipetou 300 µL</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Platí pro kroky</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>A1+B1</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>IN_TUBES – vzorky: 2 holdery po 96 Eppendorf 1,5 mL nebo QIAGEN 2,0 mL (dvojslotová svislá dvojice)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>stejné</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>obě</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>96 TIPS pro vzorky</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>stejné</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>obě</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>96 TIPS pro R-primery NEBO pufry</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>stejné</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>obě</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>OUT_PLATE / MAGNETIC PLATE / IN_PLATE (PCR 200 µL, chlazení)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>RESERVOIRS</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>obě</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>96_R-PRIMERS (PCR 200 µL, chlazení) nebo OUT_PLATE (PCR 200 µL, chlazení)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>RESERVOIRS</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>obě</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>WASTE</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>stejné</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>obě</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>8 F-PRIMERS + MM mix (pro 1 plate)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>stejné</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>obě</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Alkalický / neutralizační pufr (pro 1 plate)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>stejné</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>obě</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>C1–C3</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>L / R</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr"/>
+      <c r="C11" s="4" t="inlineStr"/>
+      <c r="D11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n"/>
+      <c r="B12" s="4" t="n"/>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="4" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n"/>
+      <c r="B13" s="4" t="n"/>
+      <c r="C13" s="4" t="n"/>
+      <c r="D13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n"/>
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n"/>
+      <c r="B15" s="4" t="n"/>
+      <c r="C15" s="4" t="n"/>
+      <c r="D15" s="4" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n"/>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="n"/>
+    </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>přesnost (precision) = náhodná odchylka, CV v %. Vyplňte pro každou třídu kroku (list 6).</t>
-        </is>
-      </c>
+      <c r="A17" s="3" t="n"/>
+      <c r="B17" s="4" t="n"/>
+      <c r="C17" s="4" t="n"/>
+      <c r="D17" s="4" t="n"/>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H65"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Seznam</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Zdroj (labware)</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Zdrojová jamka</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Objem µL</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Cíl (labware)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Cílová jamka</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Kanál (levý/pravý/auto)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Poznámka</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>pl1</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>samples#0</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>plate96_pcr#0</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr"/>
+      <c r="H2" s="4" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n"/>
+      <c r="B3" s="4" t="n"/>
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="4" t="n"/>
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="4" t="n"/>
+      <c r="H3" s="4" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="n"/>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="4" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n"/>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n"/>
+      <c r="B7" s="4" t="n"/>
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="4" t="n"/>
+      <c r="E7" s="4" t="n"/>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="4" t="n"/>
+      <c r="H7" s="4" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n"/>
+      <c r="B8" s="4" t="n"/>
+      <c r="C8" s="4" t="n"/>
+      <c r="D8" s="4" t="n"/>
+      <c r="E8" s="4" t="n"/>
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="4" t="n"/>
+      <c r="H8" s="4" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n"/>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="4" t="n"/>
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="4" t="n"/>
+      <c r="H9" s="4" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n"/>
+      <c r="B10" s="4" t="n"/>
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="4" t="n"/>
+      <c r="E10" s="4" t="n"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n"/>
+      <c r="B11" s="4" t="n"/>
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="4" t="n"/>
+      <c r="E11" s="4" t="n"/>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="4" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n"/>
+      <c r="B12" s="4" t="n"/>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="4" t="n"/>
+      <c r="E12" s="4" t="n"/>
+      <c r="F12" s="4" t="n"/>
+      <c r="G12" s="4" t="n"/>
+      <c r="H12" s="4" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n"/>
+      <c r="B13" s="4" t="n"/>
+      <c r="C13" s="4" t="n"/>
+      <c r="D13" s="4" t="n"/>
+      <c r="E13" s="4" t="n"/>
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="4" t="n"/>
+      <c r="H13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n"/>
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="n"/>
+      <c r="E14" s="4" t="n"/>
+      <c r="F14" s="4" t="n"/>
+      <c r="G14" s="4" t="n"/>
+      <c r="H14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n"/>
+      <c r="B15" s="4" t="n"/>
+      <c r="C15" s="4" t="n"/>
+      <c r="D15" s="4" t="n"/>
+      <c r="E15" s="4" t="n"/>
+      <c r="F15" s="4" t="n"/>
+      <c r="G15" s="4" t="n"/>
+      <c r="H15" s="4" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n"/>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="n"/>
+      <c r="E16" s="4" t="n"/>
+      <c r="F16" s="4" t="n"/>
+      <c r="G16" s="4" t="n"/>
+      <c r="H16" s="4" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n"/>
+      <c r="B17" s="4" t="n"/>
+      <c r="C17" s="4" t="n"/>
+      <c r="D17" s="4" t="n"/>
+      <c r="E17" s="4" t="n"/>
+      <c r="F17" s="4" t="n"/>
+      <c r="G17" s="4" t="n"/>
+      <c r="H17" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n"/>
+      <c r="B18" s="4" t="n"/>
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
+      <c r="E18" s="4" t="n"/>
+      <c r="F18" s="4" t="n"/>
+      <c r="G18" s="4" t="n"/>
+      <c r="H18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n"/>
+      <c r="B19" s="4" t="n"/>
+      <c r="C19" s="4" t="n"/>
+      <c r="D19" s="4" t="n"/>
+      <c r="E19" s="4" t="n"/>
+      <c r="F19" s="4" t="n"/>
+      <c r="G19" s="4" t="n"/>
+      <c r="H19" s="4" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n"/>
+      <c r="B20" s="4" t="n"/>
+      <c r="C20" s="4" t="n"/>
+      <c r="D20" s="4" t="n"/>
+      <c r="E20" s="4" t="n"/>
+      <c r="F20" s="4" t="n"/>
+      <c r="G20" s="4" t="n"/>
+      <c r="H20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n"/>
+      <c r="B21" s="4" t="n"/>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="n"/>
+      <c r="G21" s="4" t="n"/>
+      <c r="H21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n"/>
+      <c r="B22" s="4" t="n"/>
+      <c r="C22" s="4" t="n"/>
+      <c r="D22" s="4" t="n"/>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n"/>
+      <c r="B23" s="4" t="n"/>
+      <c r="C23" s="4" t="n"/>
+      <c r="D23" s="4" t="n"/>
+      <c r="E23" s="4" t="n"/>
+      <c r="F23" s="4" t="n"/>
+      <c r="G23" s="4" t="n"/>
+      <c r="H23" s="4" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n"/>
+      <c r="B24" s="4" t="n"/>
+      <c r="C24" s="4" t="n"/>
+      <c r="D24" s="4" t="n"/>
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="4" t="n"/>
+      <c r="G24" s="4" t="n"/>
+      <c r="H24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n"/>
+      <c r="B25" s="4" t="n"/>
+      <c r="C25" s="4" t="n"/>
+      <c r="D25" s="4" t="n"/>
+      <c r="E25" s="4" t="n"/>
+      <c r="F25" s="4" t="n"/>
+      <c r="G25" s="4" t="n"/>
+      <c r="H25" s="4" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n"/>
+      <c r="B26" s="4" t="n"/>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="n"/>
+      <c r="G26" s="4" t="n"/>
+      <c r="H26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n"/>
+      <c r="B27" s="4" t="n"/>
+      <c r="C27" s="4" t="n"/>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="4" t="n"/>
+      <c r="F27" s="4" t="n"/>
+      <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n"/>
+      <c r="B28" s="4" t="n"/>
+      <c r="C28" s="4" t="n"/>
+      <c r="D28" s="4" t="n"/>
+      <c r="E28" s="4" t="n"/>
+      <c r="F28" s="4" t="n"/>
+      <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n"/>
+      <c r="B29" s="4" t="n"/>
+      <c r="C29" s="4" t="n"/>
+      <c r="D29" s="4" t="n"/>
+      <c r="E29" s="4" t="n"/>
+      <c r="F29" s="4" t="n"/>
+      <c r="G29" s="4" t="n"/>
+      <c r="H29" s="4" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n"/>
+      <c r="B30" s="4" t="n"/>
+      <c r="C30" s="4" t="n"/>
+      <c r="D30" s="4" t="n"/>
+      <c r="E30" s="4" t="n"/>
+      <c r="F30" s="4" t="n"/>
+      <c r="G30" s="4" t="n"/>
+      <c r="H30" s="4" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n"/>
+      <c r="B31" s="4" t="n"/>
+      <c r="C31" s="4" t="n"/>
+      <c r="D31" s="4" t="n"/>
+      <c r="E31" s="4" t="n"/>
+      <c r="F31" s="4" t="n"/>
+      <c r="G31" s="4" t="n"/>
+      <c r="H31" s="4" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n"/>
+      <c r="B32" s="4" t="n"/>
+      <c r="C32" s="4" t="n"/>
+      <c r="D32" s="4" t="n"/>
+      <c r="E32" s="4" t="n"/>
+      <c r="F32" s="4" t="n"/>
+      <c r="G32" s="4" t="n"/>
+      <c r="H32" s="4" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n"/>
+      <c r="B33" s="4" t="n"/>
+      <c r="C33" s="4" t="n"/>
+      <c r="D33" s="4" t="n"/>
+      <c r="E33" s="4" t="n"/>
+      <c r="F33" s="4" t="n"/>
+      <c r="G33" s="4" t="n"/>
+      <c r="H33" s="4" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n"/>
+      <c r="B34" s="4" t="n"/>
+      <c r="C34" s="4" t="n"/>
+      <c r="D34" s="4" t="n"/>
+      <c r="E34" s="4" t="n"/>
+      <c r="F34" s="4" t="n"/>
+      <c r="G34" s="4" t="n"/>
+      <c r="H34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n"/>
+      <c r="B35" s="4" t="n"/>
+      <c r="C35" s="4" t="n"/>
+      <c r="D35" s="4" t="n"/>
+      <c r="E35" s="4" t="n"/>
+      <c r="F35" s="4" t="n"/>
+      <c r="G35" s="4" t="n"/>
+      <c r="H35" s="4" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n"/>
+      <c r="B36" s="4" t="n"/>
+      <c r="C36" s="4" t="n"/>
+      <c r="D36" s="4" t="n"/>
+      <c r="E36" s="4" t="n"/>
+      <c r="F36" s="4" t="n"/>
+      <c r="G36" s="4" t="n"/>
+      <c r="H36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n"/>
+      <c r="B37" s="4" t="n"/>
+      <c r="C37" s="4" t="n"/>
+      <c r="D37" s="4" t="n"/>
+      <c r="E37" s="4" t="n"/>
+      <c r="F37" s="4" t="n"/>
+      <c r="G37" s="4" t="n"/>
+      <c r="H37" s="4" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="n"/>
+      <c r="B38" s="4" t="n"/>
+      <c r="C38" s="4" t="n"/>
+      <c r="D38" s="4" t="n"/>
+      <c r="E38" s="4" t="n"/>
+      <c r="F38" s="4" t="n"/>
+      <c r="G38" s="4" t="n"/>
+      <c r="H38" s="4" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n"/>
+      <c r="B39" s="4" t="n"/>
+      <c r="C39" s="4" t="n"/>
+      <c r="D39" s="4" t="n"/>
+      <c r="E39" s="4" t="n"/>
+      <c r="F39" s="4" t="n"/>
+      <c r="G39" s="4" t="n"/>
+      <c r="H39" s="4" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="n"/>
+      <c r="B40" s="4" t="n"/>
+      <c r="C40" s="4" t="n"/>
+      <c r="D40" s="4" t="n"/>
+      <c r="E40" s="4" t="n"/>
+      <c r="F40" s="4" t="n"/>
+      <c r="G40" s="4" t="n"/>
+      <c r="H40" s="4" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n"/>
+      <c r="B41" s="4" t="n"/>
+      <c r="C41" s="4" t="n"/>
+      <c r="D41" s="4" t="n"/>
+      <c r="E41" s="4" t="n"/>
+      <c r="F41" s="4" t="n"/>
+      <c r="G41" s="4" t="n"/>
+      <c r="H41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n"/>
+      <c r="B42" s="4" t="n"/>
+      <c r="C42" s="4" t="n"/>
+      <c r="D42" s="4" t="n"/>
+      <c r="E42" s="4" t="n"/>
+      <c r="F42" s="4" t="n"/>
+      <c r="G42" s="4" t="n"/>
+      <c r="H42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="n"/>
+      <c r="B43" s="4" t="n"/>
+      <c r="C43" s="4" t="n"/>
+      <c r="D43" s="4" t="n"/>
+      <c r="E43" s="4" t="n"/>
+      <c r="F43" s="4" t="n"/>
+      <c r="G43" s="4" t="n"/>
+      <c r="H43" s="4" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n"/>
+      <c r="B44" s="4" t="n"/>
+      <c r="C44" s="4" t="n"/>
+      <c r="D44" s="4" t="n"/>
+      <c r="E44" s="4" t="n"/>
+      <c r="F44" s="4" t="n"/>
+      <c r="G44" s="4" t="n"/>
+      <c r="H44" s="4" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n"/>
+      <c r="B45" s="4" t="n"/>
+      <c r="C45" s="4" t="n"/>
+      <c r="D45" s="4" t="n"/>
+      <c r="E45" s="4" t="n"/>
+      <c r="F45" s="4" t="n"/>
+      <c r="G45" s="4" t="n"/>
+      <c r="H45" s="4" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="n"/>
+      <c r="B46" s="4" t="n"/>
+      <c r="C46" s="4" t="n"/>
+      <c r="D46" s="4" t="n"/>
+      <c r="E46" s="4" t="n"/>
+      <c r="F46" s="4" t="n"/>
+      <c r="G46" s="4" t="n"/>
+      <c r="H46" s="4" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="n"/>
+      <c r="B47" s="4" t="n"/>
+      <c r="C47" s="4" t="n"/>
+      <c r="D47" s="4" t="n"/>
+      <c r="E47" s="4" t="n"/>
+      <c r="F47" s="4" t="n"/>
+      <c r="G47" s="4" t="n"/>
+      <c r="H47" s="4" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="n"/>
+      <c r="B48" s="4" t="n"/>
+      <c r="C48" s="4" t="n"/>
+      <c r="D48" s="4" t="n"/>
+      <c r="E48" s="4" t="n"/>
+      <c r="F48" s="4" t="n"/>
+      <c r="G48" s="4" t="n"/>
+      <c r="H48" s="4" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n"/>
+      <c r="B49" s="4" t="n"/>
+      <c r="C49" s="4" t="n"/>
+      <c r="D49" s="4" t="n"/>
+      <c r="E49" s="4" t="n"/>
+      <c r="F49" s="4" t="n"/>
+      <c r="G49" s="4" t="n"/>
+      <c r="H49" s="4" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="n"/>
+      <c r="B50" s="4" t="n"/>
+      <c r="C50" s="4" t="n"/>
+      <c r="D50" s="4" t="n"/>
+      <c r="E50" s="4" t="n"/>
+      <c r="F50" s="4" t="n"/>
+      <c r="G50" s="4" t="n"/>
+      <c r="H50" s="4" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="n"/>
+      <c r="B51" s="4" t="n"/>
+      <c r="C51" s="4" t="n"/>
+      <c r="D51" s="4" t="n"/>
+      <c r="E51" s="4" t="n"/>
+      <c r="F51" s="4" t="n"/>
+      <c r="G51" s="4" t="n"/>
+      <c r="H51" s="4" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="n"/>
+      <c r="B52" s="4" t="n"/>
+      <c r="C52" s="4" t="n"/>
+      <c r="D52" s="4" t="n"/>
+      <c r="E52" s="4" t="n"/>
+      <c r="F52" s="4" t="n"/>
+      <c r="G52" s="4" t="n"/>
+      <c r="H52" s="4" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="n"/>
+      <c r="B53" s="4" t="n"/>
+      <c r="C53" s="4" t="n"/>
+      <c r="D53" s="4" t="n"/>
+      <c r="E53" s="4" t="n"/>
+      <c r="F53" s="4" t="n"/>
+      <c r="G53" s="4" t="n"/>
+      <c r="H53" s="4" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="n"/>
+      <c r="B54" s="4" t="n"/>
+      <c r="C54" s="4" t="n"/>
+      <c r="D54" s="4" t="n"/>
+      <c r="E54" s="4" t="n"/>
+      <c r="F54" s="4" t="n"/>
+      <c r="G54" s="4" t="n"/>
+      <c r="H54" s="4" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="n"/>
+      <c r="B55" s="4" t="n"/>
+      <c r="C55" s="4" t="n"/>
+      <c r="D55" s="4" t="n"/>
+      <c r="E55" s="4" t="n"/>
+      <c r="F55" s="4" t="n"/>
+      <c r="G55" s="4" t="n"/>
+      <c r="H55" s="4" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="n"/>
+      <c r="B56" s="4" t="n"/>
+      <c r="C56" s="4" t="n"/>
+      <c r="D56" s="4" t="n"/>
+      <c r="E56" s="4" t="n"/>
+      <c r="F56" s="4" t="n"/>
+      <c r="G56" s="4" t="n"/>
+      <c r="H56" s="4" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="n"/>
+      <c r="B57" s="4" t="n"/>
+      <c r="C57" s="4" t="n"/>
+      <c r="D57" s="4" t="n"/>
+      <c r="E57" s="4" t="n"/>
+      <c r="F57" s="4" t="n"/>
+      <c r="G57" s="4" t="n"/>
+      <c r="H57" s="4" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="n"/>
+      <c r="B58" s="4" t="n"/>
+      <c r="C58" s="4" t="n"/>
+      <c r="D58" s="4" t="n"/>
+      <c r="E58" s="4" t="n"/>
+      <c r="F58" s="4" t="n"/>
+      <c r="G58" s="4" t="n"/>
+      <c r="H58" s="4" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="n"/>
+      <c r="B59" s="4" t="n"/>
+      <c r="C59" s="4" t="n"/>
+      <c r="D59" s="4" t="n"/>
+      <c r="E59" s="4" t="n"/>
+      <c r="F59" s="4" t="n"/>
+      <c r="G59" s="4" t="n"/>
+      <c r="H59" s="4" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="n"/>
+      <c r="B60" s="4" t="n"/>
+      <c r="C60" s="4" t="n"/>
+      <c r="D60" s="4" t="n"/>
+      <c r="E60" s="4" t="n"/>
+      <c r="F60" s="4" t="n"/>
+      <c r="G60" s="4" t="n"/>
+      <c r="H60" s="4" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="n"/>
+      <c r="B61" s="4" t="n"/>
+      <c r="C61" s="4" t="n"/>
+      <c r="D61" s="4" t="n"/>
+      <c r="E61" s="4" t="n"/>
+      <c r="F61" s="4" t="n"/>
+      <c r="G61" s="4" t="n"/>
+      <c r="H61" s="4" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="n"/>
+      <c r="B62" s="4" t="n"/>
+      <c r="C62" s="4" t="n"/>
+      <c r="D62" s="4" t="n"/>
+      <c r="E62" s="4" t="n"/>
+      <c r="F62" s="4" t="n"/>
+      <c r="G62" s="4" t="n"/>
+      <c r="H62" s="4" t="n"/>
+    </row>
+    <row r="63"/>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Cherry-picking / pooling / repliky: libovolný seznam přenosů. Plánovač seskupí přenosy do vícekanálových pohybů, pokud jamky sedí na rozteči 9 mm, jinak použije 1 (krajní) kanál.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Pooling = více zdrojů do 1 cílové jamky (nová špička na zdroj, pokud se špička dotýká kapaliny); repliky = 1 zdroj do více cílů.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="G2:G262" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"auto,levý krajní,pravý krajní,libovolný 1 kanál"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -595,7 +1603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -680,203 +1688,215 @@
           <t>Osa řady kanálů vůči decku</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>podél X (zleva doprava) – odvozeno z boční pozice 'levý/pravý kanál' a SBS na výšku</t>
+        </is>
+      </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>podél X (zleva doprava) / podél Y (zepředu dozadu)</t>
+          <t>podél X / podél Y</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>KLÍČOVÉ: úzký slot max. 2 řady – 8 kanálů se tam vejde jen při ose podél X</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr"/>
+          <t>potvrdit; sloupec 96w destičky (A–H) leží podél X, 8 kanálů se vejde do úzké řady 1×8 zkumavek</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>podél X</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Rozteč kanálů (min / max)</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr"/>
+          <t>Boční pozice L/R – které kanály dosáhnou</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>jen krajní kanál (levý pro L, pravý pro R)</t>
+        </is>
+      </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>mm (9 / 4,5 / 9–19,8 …)</t>
+          <t>kanál č. / všechny</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>zarovnání na 96/384 formát</t>
+          <t>cherry-picking a odběr z vakutejnerů, 15/50 mL, Eppendorf</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>krajní</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Rozsah pipety / pipet (viz list 8)</t>
+          <t>Jednotlivé kanály: lze nasadit špičku jen na vybrané kanály (maska)?</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr"/>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>µL min–max</t>
+          <t>ano / ne / jen krajní</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>horní mez = max. nasátý objem na špičku (ne jmenovitý objem špičky)</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr"/>
+          <t>cherry-picking, pooling, částečné sloupce</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Pracovní okno přesnosti</t>
+          <t>Výměna pipety mezi konfiguracemi (12,5 µL ⇄ 300 µL)</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr"/>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>např. ≥ 10 % max. objemu pipety</t>
+          <t>ruční / automatická / hlava výměnná</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>pod tím se krok nesmí dělat touto pipetou</t>
+          <t>počet zásahů obsluhy za run; kdy se mění konfigurace A3/B3</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>≥10 % max.</t>
+          <t>ruční</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Dispense režimy podporované hlavou</t>
+          <t>Rozteč kanálů (min / max)</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr"/>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>forward / reverse / multi-dispense (repeat) / blow-out / mix / touch-off / air-gap / pre-wet</t>
+          <t>mm (9 / 4,5 / 9–19,8 …)</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>řídí, co smí plánovač použít</t>
+          <t>9 mm hlava na 384 destičce = každý 2. řádek, 4 průchody; 4,5 mm hlava = celý sloupec</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>forward, reverse, multi, mix</t>
+          <t>9</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Multi-dispense: minimální/typický přebytek</t>
+          <t>Rozsah pipety / pipet (viz list 8)</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr"/>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>µL na kanál</t>
+          <t>µL min–max</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>ztráty a počet dávek na 1 nasátí</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
+          <t>horní mez = max. nasátý objem na špičku (ne jmenovitý objem špičky)</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Prime/zahozená první dávka</t>
+          <t>Pracovní okno přesnosti</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr"/>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>ano / ne</t>
+          <t>např. ≥ 10 % max. objemu pipety</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>zpřesňuje první dávku při multi-dispense</t>
+          <t>pod tím se krok nesmí dělat touto pipetou</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>ne</t>
+          <t>≥10 % max.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Detekce hladiny (LLD)</t>
+          <t>Dispense režimy podporované hlavou</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr"/>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>ano / ne / kapacitní / tlaková</t>
+          <t>forward / reverse / multi-dispense (repeat) / blow-out / mix / touch-off / air-gap / pre-wet</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>bezkontaktní dávkování a nasávání z nízkých objemů</t>
+          <t>řídí, co smí plánovač použít</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>ne</t>
+          <t>forward, reverse, multi, mix</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Dispense: kontakt se stěnou/hladinou</t>
+          <t>Multi-dispense: minimální/typický přebytek</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr"/>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>air / wall-touch / liquid-contact – které jsou řiditelné</t>
+          <t>µL na kanál</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>pravidla znovupoužití špičky</t>
+          <t>ztráty a počet dávek na 1 nasátí</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>air, wall-touch</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Vrácení špičky do racku (tip return)</t>
+          <t>Prime/zahozená první dávka</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr"/>
@@ -887,110 +1907,114 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>umožní znovupoužití špiček mezi runy a úsporu špiček</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr"/>
+          <t>zpřesňuje první dávku při multi-dispense</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Odpad špiček – poloha</t>
+          <t>Detekce hladiny (LLD)</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr"/>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>souřadnice nebo slot</t>
+          <t>ano / ne / kapacitní / tlaková</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>dráha eject</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr"/>
+          <t>bezkontaktní dávkování a nasávání z nízkých objemů</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Rychlosti pohybu X / Y / Z</t>
+          <t>Dispense: kontakt se stěnou/hladinou</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr"/>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>mm/s</t>
+          <t>air / wall-touch / liquid-contact – které jsou řiditelné</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>model času a minimalizace pohybů</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr"/>
+          <t>pravidla znovupoužití špičky</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>air, wall-touch</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Doba nasazení / vyhození špičky</t>
+          <t>Vrácení špičky do racku (tip return)</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr"/>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>ano / ne</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>model času</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>3 / 2</t>
-        </is>
-      </c>
+          <t>umožní znovupoužití špiček mezi runy a úsporu špiček</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Průtoky nasátí / dávkování (min–max)</t>
+          <t>Odpad špiček – poloha</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr"/>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>µL/s</t>
+          <t>souřadnice nebo slot</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>model času, vazkost</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
+          <t>dráha eject</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Maximální výška labware na decku</t>
+          <t>Rychlosti pohybu X / Y / Z</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr"/>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>mm/s</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>kolize hlavy</t>
+          <t>model času a minimalizace pohybů</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr"/>
@@ -998,71 +2022,136 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Moduly na decku (třepačka, ohřev, chlazení, magnet)</t>
+          <t>Doba nasazení / vyhození špičky</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr"/>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>seznam + sloty</t>
+          <t>s</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>zabírají sloty</t>
+          <t>model času</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>žádné</t>
+          <t>3 / 2</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Vzorkové racky 96× Eppendorf – zabírají 2 sloty</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>2 sousední hlavní sloty, vodorovně?</t>
-        </is>
-      </c>
+          <t>Průtoky nasátí / dávkování (min–max)</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr"/>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>vodorovně / svisle</t>
+          <t>µL/s</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>povolená poloha</t>
+          <t>model času, vazkost</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>vodorovně</t>
+          <t>100</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Typ špiček (ClipTip) a balení</t>
+          <t>Maximální výška labware na decku</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr"/>
       <c r="C21" s="3" t="inlineStr">
         <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>kolize hlavy</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Moduly na decku (třepačka, ohřev, chlazení, magnet)</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr"/>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>seznam + sloty</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>zabírají sloty</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>žádné</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Vzorkové racky 96× Eppendorf – zabírají 2 sloty</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>A1+B1 (svisle) – dle tabulky zákazníka</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>svisle (A+B) / vodorovně</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>povolená poloha dvojslotové položky</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>svisle</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Typ špiček (ClipTip) a balení</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
           <t>12,5 / 200 / 300 / 1250 / 1000 / 384×; rack 96 nebo 384</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>kapacita racků na decku</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1075,19 +2164,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1118,7 +2207,7 @@
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>Střed X mm (od počátku robota)</t>
+          <t>Střed X mm (od středu decku)</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
@@ -1128,12 +2217,12 @@
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>Dosah všemi kanály?</t>
+          <t>Kotvení</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>Max. výška labware mm</t>
+          <t>Dosah kanály</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
@@ -1145,396 +2234,559 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>hlavní SBS</t>
+          <t>hlavní SBS (na výšku)</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>přední řada</t>
+          <t>přední hlavní řada</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
+        <v>85.48</v>
+      </c>
+      <c r="E2" s="3" t="n">
         <v>127.76</v>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>85.48</v>
       </c>
       <c r="F2" s="4" t="inlineStr"/>
       <c r="G2" s="4" t="inlineStr"/>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>ano</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr"/>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>3 šrouby do trojúhelníku</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>všech 8 kanálů</t>
+        </is>
+      </c>
       <c r="J2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>hlavní SBS</t>
+          <t>hlavní SBS (na výšku)</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>přední řada</t>
+          <t>přední hlavní řada</t>
         </is>
       </c>
       <c r="D3" s="5" t="n">
+        <v>85.48</v>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>127.76</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>85.48</v>
       </c>
       <c r="F3" s="4" t="inlineStr"/>
       <c r="G3" s="4" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>ano</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>3 šrouby do trojúhelníku</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>všech 8 kanálů</t>
+        </is>
+      </c>
       <c r="J3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>hlavní SBS</t>
+          <t>hlavní SBS (na výšku)</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>přední řada</t>
+          <t>přední hlavní řada</t>
         </is>
       </c>
       <c r="D4" s="5" t="n">
+        <v>85.48</v>
+      </c>
+      <c r="E4" s="3" t="n">
         <v>127.76</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>85.48</v>
       </c>
       <c r="F4" s="4" t="inlineStr"/>
       <c r="G4" s="4" t="inlineStr"/>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>ano</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>3 šrouby do trojúhelníku</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>všech 8 kanálů</t>
+        </is>
+      </c>
       <c r="J4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>hlavní SBS</t>
+          <t>hlavní SBS (na výšku)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>zadní řada</t>
+          <t>zadní hlavní řada</t>
         </is>
       </c>
       <c r="D5" s="5" t="n">
+        <v>85.48</v>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>127.76</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>85.48</v>
       </c>
       <c r="F5" s="4" t="inlineStr"/>
       <c r="G5" s="4" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>ano</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>3 šrouby do trojúhelníku</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>všech 8 kanálů</t>
+        </is>
+      </c>
       <c r="J5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>hlavní SBS</t>
+          <t>hlavní SBS (na výšku)</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>zadní řada</t>
+          <t>zadní hlavní řada</t>
         </is>
       </c>
       <c r="D6" s="5" t="n">
+        <v>85.48</v>
+      </c>
+      <c r="E6" s="3" t="n">
         <v>127.76</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>85.48</v>
       </c>
       <c r="F6" s="4" t="inlineStr"/>
       <c r="G6" s="4" t="inlineStr"/>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>ano</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>3 šrouby do trojúhelníku</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>všech 8 kanálů</t>
+        </is>
+      </c>
       <c r="J6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>M6</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>hlavní SBS</t>
+          <t>hlavní SBS (na výšku)</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>zadní řada</t>
+          <t>zadní hlavní řada</t>
         </is>
       </c>
       <c r="D7" s="5" t="n">
+        <v>85.48</v>
+      </c>
+      <c r="E7" s="3" t="n">
         <v>127.76</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>85.48</v>
       </c>
       <c r="F7" s="4" t="inlineStr"/>
       <c r="G7" s="4" t="inlineStr"/>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>ano</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>3 šrouby do trojúhelníku</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>všech 8 kanálů</t>
+        </is>
+      </c>
       <c r="J7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>úzký</t>
+          <t>úzký (max. 2 řady)</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>přední úzká (předsazená)</t>
+          <t>zadní úzká řada – v tabulce zákazníka chybí</t>
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>127.76</v>
-      </c>
-      <c r="E8" s="4" t="inlineStr"/>
+        <v>85.5</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>≈27–30</t>
+        </is>
+      </c>
       <c r="F8" s="4" t="inlineStr"/>
       <c r="G8" s="4" t="inlineStr"/>
-      <c r="H8" s="4" t="inlineStr"/>
-      <c r="I8" s="4" t="inlineStr"/>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>3 šrouby v řadě (rozteč 128 mm), společné pro C1–C3</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr"/>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>max. 2 řady</t>
+          <t>doplnit využití</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>úzký</t>
+          <t>úzký (max. 2 řady)</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>přední úzká (předsazená)</t>
+          <t>zadní úzká řada – v tabulce zákazníka chybí</t>
         </is>
       </c>
       <c r="D9" s="5" t="n">
-        <v>127.76</v>
-      </c>
-      <c r="E9" s="4" t="inlineStr"/>
+        <v>85.5</v>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>≈27–30</t>
+        </is>
+      </c>
       <c r="F9" s="4" t="inlineStr"/>
       <c r="G9" s="4" t="inlineStr"/>
-      <c r="H9" s="4" t="inlineStr"/>
-      <c r="I9" s="4" t="inlineStr"/>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>3 šrouby v řadě (rozteč 128 mm), společné pro C1–C3</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr"/>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>max. 2 řady</t>
+          <t>doplnit využití</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>úzký</t>
+          <t>úzký (max. 2 řady)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>přední úzká (předsazená)</t>
+          <t>zadní úzká řada – v tabulce zákazníka chybí</t>
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>127.76</v>
-      </c>
-      <c r="E10" s="4" t="inlineStr"/>
+        <v>85.5</v>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>≈27–30</t>
+        </is>
+      </c>
       <c r="F10" s="4" t="inlineStr"/>
       <c r="G10" s="4" t="inlineStr"/>
-      <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" s="4" t="inlineStr"/>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>3 šrouby v řadě (rozteč 128 mm), společné pro C1–C3</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr"/>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>max. 2 řady</t>
+          <t>doplnit využití</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>úzký</t>
+          <t>úzký (max. 2 řady)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>zadní úzká</t>
+          <t>přední úzká řada</t>
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>127.76</v>
-      </c>
-      <c r="E11" s="4" t="inlineStr"/>
+        <v>85.5</v>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>≈27</t>
+        </is>
+      </c>
       <c r="F11" s="4" t="inlineStr"/>
       <c r="G11" s="4" t="inlineStr"/>
-      <c r="H11" s="4" t="inlineStr"/>
-      <c r="I11" s="4" t="inlineStr"/>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>3 šrouby v řadě (rozteč 128 mm), společné pro 1–3</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>8 kanálů u řady 1×8 podél X</t>
+        </is>
+      </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>max. 2 řady</t>
+          <t>tabulka: WASTE / 8 F-PRIMERS + MM / pufr</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>úzký</t>
+          <t>úzký (max. 2 řady)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>zadní úzká</t>
+          <t>přední úzká řada</t>
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>127.76</v>
-      </c>
-      <c r="E12" s="4" t="inlineStr"/>
+        <v>85.5</v>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>≈27</t>
+        </is>
+      </c>
       <c r="F12" s="4" t="inlineStr"/>
       <c r="G12" s="4" t="inlineStr"/>
-      <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="4" t="inlineStr"/>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>3 šrouby v řadě (rozteč 128 mm), společné pro 1–3</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>8 kanálů u řady 1×8 podél X</t>
+        </is>
+      </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>max. 2 řady</t>
+          <t>tabulka: WASTE / 8 F-PRIMERS + MM / pufr</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>úzký</t>
+          <t>úzký (max. 2 řady)</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>zadní úzká</t>
+          <t>přední úzká řada</t>
         </is>
       </c>
       <c r="D13" s="5" t="n">
-        <v>127.76</v>
-      </c>
-      <c r="E13" s="4" t="inlineStr"/>
+        <v>85.5</v>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>≈27</t>
+        </is>
+      </c>
       <c r="F13" s="4" t="inlineStr"/>
       <c r="G13" s="4" t="inlineStr"/>
-      <c r="H13" s="4" t="inlineStr"/>
-      <c r="I13" s="4" t="inlineStr"/>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>3 šrouby v řadě (rozteč 128 mm), společné pro 1–3</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>8 kanálů u řady 1×8 podél X</t>
+        </is>
+      </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>max. 2 řady</t>
+          <t>tabulka: WASTE / 8 F-PRIMERS + MM / pufr</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>(?)</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>předsazená řada – upřesnit</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr"/>
-      <c r="D14" s="3" t="inlineStr"/>
-      <c r="E14" s="4" t="inlineStr"/>
+          <t>boční pozice</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>levý okraj</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>≈64</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>≈256 (3 šrouby, rozteč 128 mm)</t>
+        </is>
+      </c>
       <c r="F14" s="4" t="inlineStr"/>
       <c r="G14" s="4" t="inlineStr"/>
-      <c r="H14" s="4" t="inlineStr"/>
-      <c r="I14" s="4" t="inlineStr"/>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>3 šrouby v řadě podél Y</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>jen krajní kanál</t>
+        </is>
+      </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>popište/načrtněte: kolik pozic, o kolik mm je předsazena, v jakém rozsahu dosáhne hlava</t>
+          <t>vakutejnery, 15/50 mL, Eppendorf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>boční pozice</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>pravý okraj</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>≈64</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>≈256 (3 šrouby, rozteč 128 mm)</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr"/>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>3 šrouby v řadě podél Y</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>jen krajní kanál</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>vakutejnery, 15/50 mL, Eppendorf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Rozměry odvozeny z výkresu kotev (měřítko 0,455 mm/px při předpokladu, že hlavní sloty jsou SBS a těsně vedle sebe) – potvrdit skutečné rozměry plechu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Potvrdit: (1) která strana je přední (obsluha), (2) poloha slotu vůči trojúhelníku kotev, (3) do jakého rozsahu dosáhne hlava přes okraje (osa X/Y min–max).</t>
         </is>
       </c>
     </row>
@@ -3217,7 +4469,7 @@
       <formula1>"forward,reverse,multi-dispense,auto"</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H242" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"1,8,12,16,auto"</formula1>
+      <formula1>"1,8,12,16,levý krajní,pravý krajní,auto"</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I242" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"nová na jamku/sloupec,1 na krok (reuse),1 na reagencii napříč destičkami,1 na reagencii napříč runy (vrátit do racku),auto (dle kvality+kapaliny)"</formula1>

</xml_diff>

<commit_message>
Tip-pickup geometry, raised tip racks, pipette set, G-code grammar sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X1RNxQHa1nUuDBKRsS4C3g
</commit_message>
<xml_diff>
--- a/docs/labot_zadani_parametry.xlsx
+++ b/docs/labot_zadani_parametry.xlsx
@@ -18,6 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8_Pipety" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_Konfigurace" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Pick_list" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Prikazy_G" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -473,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -584,17 +585,24 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>11_Prikazy_G – logické operace pipety a vaše G-kódy (pořadí: blow-out → drop → confirm …)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Pojmy: správnost (trueness) = systematická odchylka od nominálního objemu v % nebo µL;</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
+        <is>
+          <t>Pojmy: správnost (trueness) = systematická odchylka od nominálního objemu v % nebo µL;</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>přesnost (precision) = náhodná odchylka, CV v %. Vyplňte pro každou třídu kroku (list 6).</t>
         </is>
@@ -1597,13 +1605,419 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Operace (logická)</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Význam</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Parametry</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Pravidla / pořadí</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Vaše G-kódy (příkaz + parametry)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Doba s / poznámka</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>pick_up_tip</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>nasazení špičky(ek) – všechny kanály nebo maska / krajní kanál</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>rack, sloupec, kanály</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>rack zvýšený; při jedné špičce odběr od kraje dovnitř</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr"/>
+      <c r="F2" s="4" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>aspirate (forward)</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>nasátí</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>objem, rychlost, výška</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>špička nasazená</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr"/>
+      <c r="F3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dispense (forward)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>vydání</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>objem, rychlost, výška</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>aspirate/dispense (reverse)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>reverse pipetting</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>objem + přebytek</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>multi-dispense</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>více dávek z jednoho nasátí</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>objem dávky, počet dávek, přebytek</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>k = ⌊(Vmax − přebytek)/v⌋</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>blow_out</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>vyfouknutí zbytku</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>VŽDY před drop_tip</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>drop_tip</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>odhození špičky stepper motorem</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr"/>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>bezprostředně po blow_out</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr"/>
+      <c r="F8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>confirm</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>vynulování pozice stepper motoru</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>kdy se posílá – doplnit</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>return_tip_to_rack</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>vrácení špičky na původní pozici v racku</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>rack, pozice</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>blow_out? rack musí být dosažitelný týmž kanálem</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>mix</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>míchání pístem</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>objem, cykly</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>move X/Y/Z</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>pojezd gantry</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>souřadnice, rychlost</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>bezpečná Z při přejezdu</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr"/>
+      <c r="F12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>pipette_swap</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>výměna pipety</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>z → na</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>vždy jen jedna pipeta; po výměně homing/confirm?</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr"/>
+      <c r="F13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>set_spacing</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Equalizer – rozteč kanálů</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>jen u roztahovací pipety</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr"/>
+      <c r="F14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n"/>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="4" t="n"/>
+      <c r="F15" s="4" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n"/>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="n"/>
+      <c r="E16" s="4" t="n"/>
+      <c r="F16" s="4" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n"/>
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="3" t="n"/>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="4" t="n"/>
+      <c r="F17" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n"/>
+      <c r="B18" s="3" t="n"/>
+      <c r="C18" s="3" t="n"/>
+      <c r="D18" s="3" t="n"/>
+      <c r="E18" s="4" t="n"/>
+      <c r="F18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n"/>
+      <c r="B19" s="3" t="n"/>
+      <c r="C19" s="3" t="n"/>
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="4" t="n"/>
+      <c r="F19" s="4" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n"/>
+      <c r="B20" s="3" t="n"/>
+      <c r="C20" s="3" t="n"/>
+      <c r="D20" s="3" t="n"/>
+      <c r="E20" s="4" t="n"/>
+      <c r="F20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n"/>
+      <c r="B21" s="3" t="n"/>
+      <c r="C21" s="3" t="n"/>
+      <c r="D21" s="3" t="n"/>
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n"/>
+      <c r="B22" s="3" t="n"/>
+      <c r="C22" s="3" t="n"/>
+      <c r="D22" s="3" t="n"/>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1646,7 +2060,11 @@
           <t>Pipetovací hlava – typ</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr"/>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>8 kanálů, osa řady podél X; fixní rozteč 9 mm i roztahovací (Equalizer)</t>
+        </is>
+      </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>1 kanál / 8 / 12 / 16 / Equalizer (nastavitelná rozteč) / jiné</t>
@@ -1665,7 +2083,11 @@
           <t>Počet pipet/hlav současně na gantry</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr"/>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>1 – vždy jen jedna, rychlá výměna</t>
+        </is>
+      </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
           <t>1 / 2 / výměna nástroje</t>
@@ -1811,7 +2233,11 @@
           <t>Rozsah pipety / pipet (viz list 8)</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr"/>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>12,5 / 300 / 1250 µL (všechny 8 kanálů)</t>
+        </is>
+      </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
           <t>µL min–max</t>
@@ -1853,7 +2279,11 @@
           <t>Dispense režimy podporované hlavou</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr"/>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>forward, reverse, multi-dispense, blow-out, vrácení špičky do racku (vlastní G-kódy pístu)</t>
+        </is>
+      </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
           <t>forward / reverse / multi-dispense (repeat) / blow-out / mix / touch-off / air-gap / pre-wet</t>
@@ -1968,7 +2398,11 @@
           <t>Vrácení špičky do racku (tip return)</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr"/>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
           <t>ano / ne</t>
@@ -2152,6 +2586,178 @@
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Drop špičky – řízení</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>stepper motor; vždy musí předcházet blow-out</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>popis</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>pevné pravidlo příkazové gramatiky (list 11)</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>blow-out → drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Příkaz Confirm</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>vynuluje pozici stepper motoru</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>kdy přesně se posílá? (po každém dropu / po nasazení / po každém pohybu pístu)</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>pořadí příkazů v kódu runu</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Tip racky: povýšení v Z</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>uprostřed (A2/B2) a zvýšené</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>výška podstavce v mm</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>jednotlivá špička levým/pravým kanálem – ostatní kanály přečnívají nad sousedy</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Délka špičky ClipTip 12,5 / 300 / 1250</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>kolizní kontrola přečnívajících kanálů bez špičky</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Odběr jednotlivých špiček z racku</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>levý kanál od jednoho kraje, pravý od druhého (od kraje dovnitř)</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>potvrdit pořadí</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>plánovač spotřeby špiček a kolizní pravidla</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Equalizer – změna rozteče</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>řízeno G-kódem / ručně; rozsah mm; doba změny s</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>krok s přenosem mezi různými rozteč. formáty</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Výměna pipety – doba a postup</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>s; nutný homing / Confirm / kalibrace?</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>řazení kroků podle pipety (minimum výměn)</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Rozsah pojezdů X / Y / Z a bezpečná Z</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>dosah na boční pozice, kolize</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5050,7 +5656,11 @@
         <v>9</v>
       </c>
       <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>ano (předpoklad)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -5110,7 +5720,11 @@
         <v>9</v>
       </c>
       <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>ano (předpoklad)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -5140,7 +5754,11 @@
         <v>9</v>
       </c>
       <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="4" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>ano (předpoklad)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -5416,7 +6034,11 @@
       <c r="G15" s="3" t="n">
         <v>14.2</v>
       </c>
-      <c r="H15" s="4" t="inlineStr"/>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>ano (předpoklad)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -5448,7 +6070,11 @@
       <c r="G16" s="3" t="n">
         <v>14.2</v>
       </c>
-      <c r="H16" s="4" t="inlineStr"/>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>ano (předpoklad)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -5480,7 +6106,11 @@
       <c r="G17" s="3" t="n">
         <v>14.2</v>
       </c>
-      <c r="H17" s="4" t="inlineStr"/>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>ano (předpoklad)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -5670,7 +6300,11 @@
         <v>1</v>
       </c>
       <c r="G23" s="3" t="inlineStr"/>
-      <c r="H23" s="4" t="inlineStr"/>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -5700,7 +6334,11 @@
         <v>1</v>
       </c>
       <c r="G24" s="3" t="inlineStr"/>
-      <c r="H24" s="4" t="inlineStr"/>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -5730,7 +6368,11 @@
         <v>1</v>
       </c>
       <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="4" t="inlineStr"/>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -5760,12 +6402,16 @@
         <v>1</v>
       </c>
       <c r="G26" s="3" t="inlineStr"/>
-      <c r="H26" s="4" t="inlineStr"/>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="H2:H226" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"ano,ne"</formula1>
+      <formula1>"ano,ano (předpoklad),ne"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fold in customer answers: confirm only after home, one pipette per run, dimensions sheet, strategic planning model
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X1RNxQHa1nUuDBKRsS4C3g
</commit_message>
<xml_diff>
--- a/docs/labot_zadani_parametry.xlsx
+++ b/docs/labot_zadani_parametry.xlsx
@@ -19,6 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_Konfigurace" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Pick_list" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Prikazy_G" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Rozmery" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -474,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -587,22 +588,29 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>11_Prikazy_G – logické operace pipety a vaše G-kódy (pořadí: blow-out → drop → confirm …)</t>
+          <t>11_Prikazy_G – logické operace pipety a vaše G-kódy (home → confirm; blow_out → drop_tip …)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>12_Rozmery   – rozměry potřebné pro výpočty (stav: známo / hypotéza / čeká)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Pojmy: správnost (trueness) = systematická odchylka od nominálního objemu v % nebo µL;</t>
-        </is>
-      </c>
+      <c r="A19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
+        <is>
+          <t>Pojmy: správnost (trueness) = systematická odchylka od nominálního objemu v % nebo µL;</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>přesnost (precision) = náhodná odchylka, CV v %. Vyplňte pro každou třídu kroku (list 6).</t>
         </is>
@@ -1820,7 +1828,7 @@
       <c r="C9" s="3" t="inlineStr"/>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>kdy se posílá – doplnit</t>
+          <t>jen na začátku běhu po Home (kontrola X, Y, Z)</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr"/>
@@ -1897,22 +1905,18 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>pipette_swap</t>
+          <t>home</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>výměna pipety</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>z → na</t>
-        </is>
-      </c>
+          <t>Home + kontrola pozice X, Y, Z</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr"/>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>vždy jen jedna pipeta; po výměně homing/confirm?</t>
+          <t>na začátku běhu, následuje confirm</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr"/>
@@ -2005,6 +2009,954 @@
       <c r="D22" s="3" t="n"/>
       <c r="E22" s="4" t="n"/>
       <c r="F22" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="56" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Skupina</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Rozměr / veličina</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Stav / hodnota</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Jednotka</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Zdroj</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>K čemu se použije ve výpočtu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Deck</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Rozteč kotev hlavních slotů ve směru X (střed trojúhelníku ↔ střed sousedního)</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>HYPOTÉZA 90 (z výkresu jen px: 187)</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>výkres kotev</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>jediné číslo dá měřítko celého výkresu; poloha všech pozic</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Deck</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Rozteč ve směru Y (A ↔ B)</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>HYPOTÉZA 135 (poměr Y/X změřen 1,50)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>výkres kotev</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>vzdálenosti přejezdů, mezera mezi plasticware</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Deck</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Trojúhelník kotev: základna × výška</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>z výkresu ≈ ½·P_x × P_x (45 × 90)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>výkres kotev</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>střed plasticware = střed trojúhelníku?</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Deck</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Úzké řady 1–3 a C1–C3: kolik pozic a kde je střed vůči 3 šroubům v řadě</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>ČEKÁ – hypotéza: každý šroub = střed jedné pozice (rozteč ≈ 135)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>ano/ne</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>tabulka + výkres</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>poloha úzkých pozic; konflikt s přední hranou A při středění na šroub</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Deck</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Boční pozice L/R: kolik pozic na stranu a střed vůči šroubům</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>ČEKÁ – hypotéza: 3 pozice na stranu, střed na šroubu (Y rozteč ≈ 135, X ≈ ±189 od středu)</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>výkres kotev</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>boční labware a dosah krajního kanálu</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Deck</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Posun pozic dopředu (housing pipety, ≈ 40 mm) a dosah bočních šroubů −20 mm</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>IGNOROVAT (zadáno)</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>zákazník</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Deck</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Mezery mezi plasticware</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>vyplývají z rozteče kotev − rozměr labware (stejná mezera v Y)</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>D1–D2, L1</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>kontrola kolizí, vycentrování na šrouby</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Stroj</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Rozsah pojezdů X / Y / Z</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>ČEKÁ (nebo v config souboru)</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>config</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>kontrola dosahu, boční pozice</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Stroj</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Home pozice a vztah k souřadnicím kotev</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>ČEKÁ (v config souboru)</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>config</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>převod pozice → G-kód souřadnice</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Stroj</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Referenční kanál pro XY (K1 / střed hlavy) a offset ostatních kanálů</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>ČEKÁ</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>config</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>poloha k-tého kanálu = ref + (k−1)·rozteč</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Stroj</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Rozteč kanálů: fixní 9 mm; Equalizer rozsah</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>fixní 9; Equalizer dle listu 8 (9–14,2 / 4,5–14,2), G-kód na separátním servu</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>list 8</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>mapování formátů 9 ↔ 14,2 mm ↔ 4,5 mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Stroj</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Délka špičky ClipTip 12,5 / 300 / 1250 (a délka kužele pipety)</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>30–120 mm dle pipety – přesně ČEKÁ</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>zákazník</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>kolizní kontrola přečnívajících kanálů</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Stroj</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Max zdvih = délka špičky + 25 mm</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>ČEKÁ: co přesně? (max. povýšení racku nad deskou / max. zdvih Z osy od pracovní hladiny)</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>zákazník</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>horní mez výšky racků špiček</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Stroj</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Bezpečná Z pro přejezdy mezi pozicemi</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>ČEKÁ (config)</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>config</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>legalita přejezdu nad vyššími labware</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Labware</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Půdorys L × W včetně holderu/racku (SBS destička 127,76 × 85,48; rack Eppendorf, deepwell, zásobník, boční držáky)</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>SBS známo; holdery ČEKÁ</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>katalog výrobce / měření</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>mezery, zakrytí kotev</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Labware</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Výška H včetně podstavce / chlazení / magnetické desky</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>ČEKÁ</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>měření</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>kolize s přečnívajícími kanály</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Labware</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Poloha jamky A1 vůči středu labware a rozteč jamek</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>SBS 9 mm standard; holdery ČEKÁ</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>katalog</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>souřadnice všech jamek</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Labware</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Tvar jamky/zkumavky: vnitřní průměr nebo průřez, hloubka, tvar dna</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>ČEKÁ (1,5 mL, 2 mL QIAGEN, PCR 200 µL, deepwell, 15/50 mL, vakutejner)</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>katalog</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>výška hladiny z objemu → bezkontaktní/kontaktní dávkování, ponor</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>L5</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Labware</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Max a mrtvý objem na jamku</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>předvyplněno v listu 3 – potvrdit</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>µL</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>list 3</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>počet nasátí, plnění zdrojů</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>L6</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Labware</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Tip rack: rozteč špiček, výška špiček nad rackem, výška podstavce h_rack na každý rack</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>rozteč 9; ostatní ČEKÁ; h_rack = výstup optimalizace</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>měření</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>odběr jednotlivých špiček, kolize</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>L7</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Labware</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Úzká řada: hloubka (≤ 2 řady), počet zkumavek v řadě (8 po 9 mm?), výška</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>ČEKÁ</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>měření</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>dosah všemi 8 kanály, nasátí z 8 primerů najednou</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>L8</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Labware</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Boční držáky: průměr a výška zkumavek (15/50 mL, vakutejner, Eppendorf), rozteč</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>ČEKÁ</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>měření</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>krajní kanál, hloubka ponoru</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Špičky</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Min / max objem pipety a špičky</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>0,5–12,5 / 10–300 / 15–1250 µL (list 8)</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>µL</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>list 8</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>volba pipety pro běh, multi-dispense počet dávek</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Špičky</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Průměr ústí špičky (ponor do jamky) a rozteč 9 mm vs 4,5 mm formát</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>ČEKÁ</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>katalog ClipTip</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>kontakt s kapalinou / stěnou, 384 destičky</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2017,7 +2969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2095,7 +3047,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>určuje, zda lze střídat rozsahy bez zásahu</t>
+          <t>jeden běh = jedna pipeta</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -2187,7 +3139,11 @@
           <t>Výměna pipety mezi konfiguracemi (12,5 µL ⇄ 300 µL)</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr"/>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>ruční, výjimečná, mimo běh</t>
+        </is>
+      </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
           <t>ruční / automatická / hlava výměnná</t>
@@ -2195,7 +3151,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>počet zásahů obsluhy za run; kdy se mění konfigurace A3/B3</t>
+          <t>konfigurace A3/B3 se mění jen mezi běhy</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -2360,7 +3316,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>bezkontaktní dávkování a nasávání z nízkých objemů</t>
+          <t>bezkontaktní dávkování – bez LLD se výška hladiny počítá z objemu a geometrie jamky</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -2610,7 +3566,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>blow-out → drop</t>
+          <t>blow_out → drop_tip</t>
         </is>
       </c>
     </row>
@@ -2622,20 +3578,24 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>vynuluje pozici stepper motoru</t>
+          <t>jen na začátku běhu po Home (kontrola pozice X, Y, Z)</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>kdy přesně se posílá? (po každém dropu / po nasazení / po každém pohybu pístu)</t>
+          <t>není součástí drop makra</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>pořadí příkazů v kódu runu</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr"/>
+          <t>gramatika příkazů</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>po Home</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -2645,12 +3605,12 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>uprostřed (A2/B2) a zvýšené</t>
+          <t>výška se liší podle rack a je optimalizovaná kvůli kolizím; max zdvih = délka špičky (30–120 mm dle pipety) + 25 mm</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>výška podstavce v mm</t>
+          <t>mm na rack (výstup optimalizace)</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -2708,10 +3668,14 @@
           <t>Equalizer – změna rozteče</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr"/>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>G-kód, samostatné servo; rozsah viz list 8</t>
+        </is>
+      </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>řízeno G-kódem / ručně; rozsah mm; doba změny s</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -2724,40 +3688,63 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Výměna pipety – doba a postup</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr"/>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>s; nutný homing / Confirm / kalibrace?</t>
-        </is>
-      </c>
+          <t>Výměna pipety</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>ruční, výjimečná – v jednom běhu se s ní nepočítá</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr"/>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>řazení kroků podle pipety (minimum výměn)</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr"/>
+          <t>jeden běh = jedna pipeta (rozsah objemů musí pokrýt všechny kroky)</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>1 pipeta / běh</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
+          <t>Rychlosti a zrychlení X/Y/Z</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>odloženo – dodá zákazník v konfiguračním souboru a pravidlech</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>strategické plánování počítá počty pohybů a vzdálenosti, ne čas</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
           <t>Rozsah pojezdů X / Y / Z a bezpečná Z</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr"/>
-      <c r="C32" s="3" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr"/>
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>dosah na boční pozice, kolize</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5279,7 +6266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -5377,79 +6364,79 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Formát destiček</t>
+          <t>Pipeta pro běh (jedna)</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr"/>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>96 / 384 / smíšené</t>
+          <t>12,5 / 300 / 1250 µL (+ fixní / Equalizer)</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>plánovač zvolí podle rozsahu objemů, pokud nezadáte</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Proměnný počet vzorků (částečné sloupce)</t>
+          <t>Formát destiček</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr"/>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>ano / ne</t>
+          <t>96 / 384 / smíšené</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>ne</t>
+          <t>96</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Dohled obsluhy – max. počet zásahů na run</t>
+          <t>Proměnný počet vzorků (částečné sloupce)</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr"/>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>počet (výměny racků apod.)</t>
+          <t>ano / ne</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>ne</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Priorita: minimum času runu</t>
+          <t>Dohled obsluhy – max. počet zásahů na run</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr"/>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>1–5</t>
+          <t>počet (výměny racků apod.)</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Priorita: minimum spotřeby špiček</t>
+          <t>Priorita: minimum času runu</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr"/>
@@ -5460,14 +6447,14 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Priorita: minimum slotů/ruční práce</t>
+          <t>Priorita: minimum spotřeby špiček</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr"/>
@@ -5478,14 +6465,14 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Priorita: minimum rizika kontaminace</t>
+          <t>Priorita: minimum slotů/ruční práce</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr"/>
@@ -5496,41 +6483,59 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Znovupoužití špiček mezi runy / směnami</t>
+          <t>Priorita: minimum rizika kontaminace</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr"/>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>ne / v rámci dne</t>
+          <t>1–5</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>ne</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Požadovaný výstup</t>
+          <t>Znovupoužití špiček mezi runy / směnami</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr"/>
       <c r="C14" s="3" t="inlineStr">
         <is>
+          <t>ne / v rámci dne</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Požadovaný výstup</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
           <t>zadání pro kód / hotový kód / protokol IQ-OQ</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>